<commit_message>
Inventário material médico: contagem única por foto, organizado por categorias com total 166 unidades
</commit_message>
<xml_diff>
--- a/Inventario_Material_Medico_FYTLOQ.xlsx
+++ b/Inventario_Material_Medico_FYTLOQ.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,6 +50,11 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -66,8 +71,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D3D3D3"/>
-        <bgColor rgb="00D3D3D3"/>
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -77,7 +82,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -91,11 +96,32 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -110,6 +136,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -119,6 +148,11 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -484,27 +518,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>INVENTÁRIO MATERIAL MÉDICO - FYTLOQ</t>
+          <t>INVENTÁRIO DE MATERIAL MÉDICO</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Data: 24/07/2026</t>
+          <t>Data: 24/07/2026  |  Contagem única (não somada entre fotos)</t>
         </is>
       </c>
     </row>
@@ -526,7 +560,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Un</t>
+          <t>Unidade</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -550,20 +584,20 @@
       <c r="A6" s="5" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Seringas Azuis</t>
+          <t>Seringas pequenas (êmbolo azul)</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>48</v>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+        <v>13</v>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>unid</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Cartelas com seringas estéreis</t>
+          <t>À direita do tablet (aprox.)</t>
         </is>
       </c>
     </row>
@@ -571,158 +605,168 @@
       <c r="A7" s="5" t="inlineStr"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Seringas Verdes</t>
+          <t>Seringas BD (transparentes)</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
+        <v>10</v>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>unid</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Cartelas com seringas estéreis</t>
+          <t>Coluna central (aprox.)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>LUVAS</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr"/>
-      <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr"/>
+      <c r="A8" s="5" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Seringas com êmbolo verde</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Coluna à esquerda (aprox.)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>DuPont Tyvek XXL</t>
+          <t>Seringas pequenas c/ agulha (laranja)</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>emb</t>
+        <v>8</v>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Embalagem completa</t>
+          <t>Canto esquerdo (aprox.)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr"/>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Luvas Nitrile Azuis</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>emb</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Embalagem completa</t>
-        </is>
-      </c>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>AGULHAS</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>BATAS</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr"/>
-      <c r="C11" s="4" t="inlineStr"/>
-      <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr"/>
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Agulhas hipodérmicas (verdes)</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Cartela de agulhas (aprox.)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr"/>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Batas DocWorld Azuis (L)</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>unid</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Tamanho L</t>
-        </is>
-      </c>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>LUVAS CIRÚRGICAS</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr"/>
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr"/>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Bata Tyvek</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="n">
+          <t>Sempermed derma PF 7.5</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>unid</t>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>par</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Proteção descartável</t>
+          <t>Estéril, embalado</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>GAZES/COMPRESSAS</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr"/>
-      <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr"/>
-      <c r="E14" s="4" t="inlineStr"/>
+      <c r="A14" s="5" t="inlineStr"/>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Sempermed supreme 8</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Estéril, embalado</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr"/>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Gazes estéreis (packs)</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>pack</t>
+          <t>Sempermed supreme 7</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>par</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Embalagens individuais</t>
+          <t>Estéril, embalado</t>
         </is>
       </c>
     </row>
@@ -730,80 +774,80 @@
       <c r="A16" s="5" t="inlineStr"/>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Compressas verdes (bandejas)</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="n">
+          <t>Gammex PI Hybrid 6½</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>bandeja</t>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>par</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Em bandeja</t>
+          <t>Ansell, estéril</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>FITAS ADESIVAS</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr"/>
-      <c r="C17" s="4" t="inlineStr"/>
-      <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="4" t="inlineStr"/>
+      <c r="A17" s="5" t="inlineStr"/>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>iNtouch Natural (látex)</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Estéril</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr"/>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Tape Médico Branco</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>rolo</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>Rolos completos</t>
-        </is>
-      </c>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>LUVAS (CAIXA)</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr"/>
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr"/>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Tape Médico Cor Pele</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>rolo</t>
+          <t>Continente Luvas Superfinas Látex S/M</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>caixa</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Rolos completos</t>
+          <t>10 unidades</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>FRASCOS/SOLUÇÕES</t>
+          <t>FATOS/BATAS</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr"/>
@@ -815,199 +859,800 @@
       <c r="A21" s="5" t="inlineStr"/>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Frascos medicinais</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
+          <t>DocWorld bata azul (L)</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>unid</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Diversos tamanhos</t>
+          <t>1 set cada, estéril</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>TUBOS</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr"/>
-      <c r="C22" s="4" t="inlineStr"/>
-      <c r="D22" s="4" t="inlineStr"/>
-      <c r="E22" s="4" t="inlineStr"/>
+      <c r="A22" s="5" t="inlineStr"/>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>DuPont Tyvek fato integral (XXL)</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Proteção CHF5a</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr"/>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Tubo Transparente</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>unid</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>Tubo enrolado</t>
-        </is>
-      </c>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>CAMPOS CIRÚRGICOS</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr"/>
+      <c r="C23" s="4" t="inlineStr"/>
+      <c r="D23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>PINÇAS/TESOURAS</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr"/>
-      <c r="C24" s="4" t="inlineStr"/>
-      <c r="D24" s="4" t="inlineStr"/>
-      <c r="E24" s="4" t="inlineStr"/>
+      <c r="A24" s="5" t="inlineStr"/>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Covrel Surgical Drape 1m x 150cm</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Bastos Viegas, estéril</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr"/>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Packs com pinça e tesoura</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>pack</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>1 pinça + 1 tesoura por pack</t>
-        </is>
-      </c>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>FIOS DE SUTURA</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr"/>
+      <c r="C25" s="4" t="inlineStr"/>
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>PROTEÇÃO CAPILAR</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr"/>
-      <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" s="4" t="inlineStr"/>
-      <c r="E26" s="4" t="inlineStr"/>
+      <c r="A26" s="5" t="inlineStr"/>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Vicryl Rapide 4-0 (W9918)</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Ethicon PC-3 (aprox.)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr"/>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Bonés Médicos</t>
+          <t>Vicryl Rapide 3-0 (W9919)</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
+        <v>6</v>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>unid</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Cor verde</t>
+          <t>Ethicon PC-3 (aprox.)</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>PENSOS/CURATIVOS</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr"/>
-      <c r="C28" s="4" t="inlineStr"/>
-      <c r="D28" s="4" t="inlineStr"/>
-      <c r="E28" s="4" t="inlineStr"/>
+      <c r="A28" s="5" t="inlineStr"/>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Vicryl Rapide 5-0 (W9969)</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Ethicon (aprox.)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr"/>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Pensos variados</t>
+          <t>Vicryl Rapide 2-0 (W9938)</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>pack</t>
+        <v>5</v>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Vários tipos e tamanhos</t>
+          <t>Ethicon (aprox.)</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>DOCUMENTAÇÃO</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr"/>
-      <c r="C30" s="4" t="inlineStr"/>
-      <c r="D30" s="4" t="inlineStr"/>
-      <c r="E30" s="4" t="inlineStr"/>
+      <c r="A30" s="5" t="inlineStr"/>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Vicryl Rapide 5-0 (W9960)</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Ethicon (aprox.)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr"/>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Folhas de Instruções</t>
+          <t>Silkam 2/0 e 4/0</t>
         </is>
       </c>
       <c r="C31" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>B.Braun (aprox.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr"/>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Dafilon 3/0</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>B.Braun</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>LÂMINAS BISTURI</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr"/>
+      <c r="C33" s="4" t="inlineStr"/>
+      <c r="D33" s="4" t="inlineStr"/>
+      <c r="E33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr"/>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Lâminas nº15 e nº11</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Cartelas estéreis (aprox.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>PENSOS/CURATIVOS</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr"/>
+      <c r="C35" s="4" t="inlineStr"/>
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr"/>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Allevyn Classic</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Smith &amp; Nephew</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr"/>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Aquacel Ag+ Extra 10x10</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Convatec</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr"/>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Primapore 10x8</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Smith &amp; Nephew (aprox.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr"/>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Jelonet 10x10 (parafina)</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Smith &amp; Nephew</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr"/>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>3M Tegaderm Film</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Penso transparente</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr"/>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>3M Steri-Strip</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Tiras de aproximação (aprox.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr"/>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Algoplaque 10x10</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Penso hidrocolóide</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr"/>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>IVALON Epistaxis Packing</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Q602310</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>LIGADURAS</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr"/>
+      <c r="C44" s="4" t="inlineStr"/>
+      <c r="D44" s="4" t="inlineStr"/>
+      <c r="E44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr"/>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Safix plus</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Ligadura</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr"/>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Peha-haft (autoaderente)</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>caixa</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Hartmann</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr"/>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Scotchcast Plus 12.7cm</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>3M, gesso sintético</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>FITAS ADESIVAS</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr"/>
+      <c r="C48" s="4" t="inlineStr"/>
+      <c r="D48" s="4" t="inlineStr"/>
+      <c r="E48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr"/>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Rolo adesivo branco</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>rolo</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Adesivo cirúrgico</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr"/>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Leukostrip (tiras aproximação)</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>pack</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Smith &amp; Nephew</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>MEDICAÇÃO</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr"/>
+      <c r="C51" s="4" t="inlineStr"/>
+      <c r="D51" s="4" t="inlineStr"/>
+      <c r="E51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr"/>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Frascos/vials de vidro</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Medicação injetável (aprox.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr"/>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Ampolas de vidro</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Medicação (aprox.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr"/>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Ampolas plástico (soro/cloreto)</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Solução (aprox.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>KITS SUTURA</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr"/>
+      <c r="C55" s="4" t="inlineStr"/>
+      <c r="D55" s="4" t="inlineStr"/>
+      <c r="E55" s="4" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr"/>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Tabuleiro c/ pinça + tesoura</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>pack</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>1 pinça + 1 tesoura cada</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>OUTROS</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr"/>
+      <c r="C57" s="4" t="inlineStr"/>
+      <c r="D57" s="4" t="inlineStr"/>
+      <c r="E57" s="4" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr"/>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Tubo transparente (drenagem)</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Enrolado</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr"/>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Toucas cirúrgicas (verdes)</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Proteção capilar (aprox.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr"/>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Wiclom (grampos/clips coloridos)</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>saco</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr"/>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Folhas de instruções/manuais</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
         <is>
           <t>lote</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Manuais diversos</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL DE ITENS</t>
-        </is>
-      </c>
-      <c r="C33" s="8">
-        <f>SUM(C5:C40)</f>
-        <v/>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Documentação</t>
+        </is>
+      </c>
+    </row>
+    <row r="62"/>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL DE UNIDADES</t>
+        </is>
+      </c>
+      <c r="B63" s="12" t="n"/>
+      <c r="C63" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="D63" s="10" t="n"/>
+      <c r="E63" s="10" t="n"/>
+    </row>
+    <row r="65" ht="45" customHeight="1">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>NOTA: Contagem feita a partir das fotografias, cada item contado uma só vez (as fotos são vários ângulos do mesmo material). Itens marcados '(aprox.)' estão empilhados ou parcialmente tapados — confirmar fisicamente. Todo o material está em embalagem estéril e original.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A33:B33"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A63:B63"/>
+    <mergeCell ref="A65:E65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lâminas de bisturi (nº24, nº22, outros) e ligadura adesiva elástica ao inventário
</commit_message>
<xml_diff>
--- a/Inventario_Material_Medico_FYTLOQ.xlsx
+++ b/Inventario_Material_Medico_FYTLOQ.xlsx
@@ -82,7 +82,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -96,32 +96,11 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -152,7 +131,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -518,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1120,25 +1098,35 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>PENSOS/CURATIVOS</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr"/>
-      <c r="C35" s="4" t="inlineStr"/>
-      <c r="D35" s="4" t="inlineStr"/>
-      <c r="E35" s="4" t="inlineStr"/>
+      <c r="A35" s="5" t="inlineStr"/>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Lâminas nº24 (embalagem azul)</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Cartelas estéreis (aprox.)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr"/>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Allevyn Classic</t>
-        </is>
-      </c>
-      <c r="C36" s="7" t="n">
-        <v>1</v>
+          <t>Lâminas nº22 (embalagem azul)</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>6</v>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
@@ -1147,7 +1135,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Smith &amp; Nephew</t>
+          <t>Cartelas estéreis (aprox.)</t>
         </is>
       </c>
     </row>
@@ -1155,11 +1143,11 @@
       <c r="A37" s="5" t="inlineStr"/>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Aquacel Ag+ Extra 10x10</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="n">
-        <v>2</v>
+          <t>Lâminas outros nº (embalagem preta)</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>14</v>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
@@ -1168,40 +1156,30 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Convatec</t>
+          <t>Cartelas estéreis (aprox.)</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr"/>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>Primapore 10x8</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D38" s="7" t="inlineStr">
-        <is>
-          <t>unid</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Smith &amp; Nephew (aprox.)</t>
-        </is>
-      </c>
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>PENSOS/CURATIVOS</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr"/>
+      <c r="C38" s="4" t="inlineStr"/>
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr"/>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Jelonet 10x10 (parafina)</t>
+          <t>Allevyn Classic</t>
         </is>
       </c>
       <c r="C39" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
@@ -1218,7 +1196,7 @@
       <c r="A40" s="5" t="inlineStr"/>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>3M Tegaderm Film</t>
+          <t>Aquacel Ag+ Extra 10x10</t>
         </is>
       </c>
       <c r="C40" s="7" t="n">
@@ -1231,7 +1209,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Penso transparente</t>
+          <t>Convatec</t>
         </is>
       </c>
     </row>
@@ -1239,11 +1217,11 @@
       <c r="A41" s="5" t="inlineStr"/>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>3M Steri-Strip</t>
+          <t>Primapore 10x8</t>
         </is>
       </c>
       <c r="C41" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
@@ -1252,7 +1230,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Tiras de aproximação (aprox.)</t>
+          <t>Smith &amp; Nephew (aprox.)</t>
         </is>
       </c>
     </row>
@@ -1260,11 +1238,11 @@
       <c r="A42" s="5" t="inlineStr"/>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Algoplaque 10x10</t>
+          <t>Jelonet 10x10 (parafina)</t>
         </is>
       </c>
       <c r="C42" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
@@ -1273,7 +1251,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>Penso hidrocolóide</t>
+          <t>Smith &amp; Nephew</t>
         </is>
       </c>
     </row>
@@ -1281,11 +1259,11 @@
       <c r="A43" s="5" t="inlineStr"/>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>IVALON Epistaxis Packing</t>
+          <t>3M Tegaderm Film</t>
         </is>
       </c>
       <c r="C43" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
@@ -1294,30 +1272,40 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Q602310</t>
+          <t>Penso transparente</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>LIGADURAS</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr"/>
-      <c r="C44" s="4" t="inlineStr"/>
-      <c r="D44" s="4" t="inlineStr"/>
-      <c r="E44" s="4" t="inlineStr"/>
+      <c r="A44" s="5" t="inlineStr"/>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>3M Steri-Strip</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Tiras de aproximação (aprox.)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr"/>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Safix plus</t>
+          <t>Algoplaque 10x10</t>
         </is>
       </c>
       <c r="C45" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
@@ -1326,7 +1314,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Ligadura</t>
+          <t>Penso hidrocolóide</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1322,7 @@
       <c r="A46" s="5" t="inlineStr"/>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Peha-haft (autoaderente)</t>
+          <t>IVALON Epistaxis Packing</t>
         </is>
       </c>
       <c r="C46" s="7" t="n">
@@ -1342,65 +1330,65 @@
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>caixa</t>
+          <t>unid</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Hartmann</t>
+          <t>Q602310</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="inlineStr"/>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>Scotchcast Plus 12.7cm</t>
-        </is>
-      </c>
-      <c r="C47" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>unid</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>3M, gesso sintético</t>
-        </is>
-      </c>
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>LIGADURAS</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr"/>
+      <c r="C47" s="4" t="inlineStr"/>
+      <c r="D47" s="4" t="inlineStr"/>
+      <c r="E47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>FITAS ADESIVAS</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr"/>
-      <c r="C48" s="4" t="inlineStr"/>
-      <c r="D48" s="4" t="inlineStr"/>
-      <c r="E48" s="4" t="inlineStr"/>
+      <c r="A48" s="5" t="inlineStr"/>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Safix plus</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Ligadura</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr"/>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Rolo adesivo branco</t>
+          <t>Peha-haft (autoaderente)</t>
         </is>
       </c>
       <c r="C49" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>rolo</t>
+          <t>caixa</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Adesivo cirúrgico</t>
+          <t>Hartmann</t>
         </is>
       </c>
     </row>
@@ -1408,73 +1396,73 @@
       <c r="A50" s="5" t="inlineStr"/>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Leukostrip (tiras aproximação)</t>
+          <t>Scotchcast Plus 12.7cm</t>
         </is>
       </c>
       <c r="C50" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>unid</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>Smith &amp; Nephew</t>
+          <t>3M, gesso sintético</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>MEDICAÇÃO</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr"/>
-      <c r="C51" s="4" t="inlineStr"/>
-      <c r="D51" s="4" t="inlineStr"/>
-      <c r="E51" s="4" t="inlineStr"/>
+      <c r="A51" s="5" t="inlineStr"/>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Ligadura adesiva elástica (óxido zinco)</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>caixa</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Elastic adhesive bandage, BV</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="inlineStr"/>
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>Frascos/vials de vidro</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D52" s="7" t="inlineStr">
-        <is>
-          <t>unid</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Medicação injetável (aprox.)</t>
-        </is>
-      </c>
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>FITAS ADESIVAS</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr"/>
+      <c r="C52" s="4" t="inlineStr"/>
+      <c r="D52" s="4" t="inlineStr"/>
+      <c r="E52" s="4" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr"/>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Ampolas de vidro</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="n">
-        <v>6</v>
+          <t>Rolo adesivo branco</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="n">
+        <v>2</v>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>unid</t>
+          <t>rolo</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>Medicação (aprox.)</t>
+          <t>Adesivo cirúrgico</t>
         </is>
       </c>
     </row>
@@ -1482,27 +1470,27 @@
       <c r="A54" s="5" t="inlineStr"/>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Ampolas plástico (soro/cloreto)</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="n">
-        <v>6</v>
+          <t>Leukostrip (tiras aproximação)</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>unid</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>Solução (aprox.)</t>
+          <t>Smith &amp; Nephew</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>KITS SUTURA</t>
+          <t>MEDICAÇÃO</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr"/>
@@ -1514,43 +1502,53 @@
       <c r="A56" s="5" t="inlineStr"/>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Tabuleiro c/ pinça + tesoura</t>
-        </is>
-      </c>
-      <c r="C56" s="7" t="n">
-        <v>2</v>
+          <t>Frascos/vials de vidro</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="n">
+        <v>4</v>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>unid</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>1 pinça + 1 tesoura cada</t>
+          <t>Medicação injetável (aprox.)</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>OUTROS</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr"/>
-      <c r="C57" s="4" t="inlineStr"/>
-      <c r="D57" s="4" t="inlineStr"/>
-      <c r="E57" s="4" t="inlineStr"/>
+      <c r="A57" s="5" t="inlineStr"/>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Ampolas de vidro</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Medicação (aprox.)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr"/>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Tubo transparente (drenagem)</t>
-        </is>
-      </c>
-      <c r="C58" s="7" t="n">
-        <v>1</v>
+          <t>Ampolas plástico (soro/cloreto)</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="n">
+        <v>6</v>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
@@ -1559,89 +1557,152 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>Enrolado</t>
+          <t>Solução (aprox.)</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="inlineStr"/>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>Toucas cirúrgicas (verdes)</t>
-        </is>
-      </c>
-      <c r="C59" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D59" s="7" t="inlineStr">
-        <is>
-          <t>unid</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Proteção capilar (aprox.)</t>
-        </is>
-      </c>
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>KITS SUTURA</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr"/>
+      <c r="C59" s="4" t="inlineStr"/>
+      <c r="D59" s="4" t="inlineStr"/>
+      <c r="E59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr"/>
       <c r="B60" s="5" t="inlineStr">
         <is>
+          <t>Tabuleiro c/ pinça + tesoura</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>pack</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>1 pinça + 1 tesoura cada</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>OUTROS</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr"/>
+      <c r="C61" s="4" t="inlineStr"/>
+      <c r="D61" s="4" t="inlineStr"/>
+      <c r="E61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr"/>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Tubo transparente (drenagem)</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Enrolado</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr"/>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>Toucas cirúrgicas (verdes)</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Proteção capilar (aprox.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr"/>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
           <t>Wiclom (grampos/clips coloridos)</t>
         </is>
       </c>
-      <c r="C60" s="7" t="n">
+      <c r="C64" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D60" s="7" t="inlineStr">
+      <c r="D64" s="7" t="inlineStr">
         <is>
           <t>saco</t>
         </is>
       </c>
-      <c r="E60" s="5" t="inlineStr">
+      <c r="E64" s="5" t="inlineStr">
         <is>
           <t>Conjunto</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr"/>
-      <c r="B61" s="5" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr"/>
+      <c r="B65" s="5" t="inlineStr">
         <is>
           <t>Folhas de instruções/manuais</t>
         </is>
       </c>
-      <c r="C61" s="7" t="n">
+      <c r="C65" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D61" s="7" t="inlineStr">
+      <c r="D65" s="7" t="inlineStr">
         <is>
           <t>lote</t>
         </is>
       </c>
-      <c r="E61" s="5" t="inlineStr">
+      <c r="E65" s="5" t="inlineStr">
         <is>
           <t>Documentação</t>
         </is>
       </c>
     </row>
-    <row r="62"/>
-    <row r="63">
-      <c r="A63" s="8" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
         <is>
           <t>TOTAL DE UNIDADES</t>
         </is>
       </c>
-      <c r="B63" s="12" t="n"/>
-      <c r="C63" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="D63" s="10" t="n"/>
-      <c r="E63" s="10" t="n"/>
-    </row>
-    <row r="65" ht="45" customHeight="1">
-      <c r="A65" s="11" t="inlineStr">
+      <c r="C67" s="9">
+        <f>SUM(C5:C65)</f>
+        <v/>
+      </c>
+      <c r="D67" s="10" t="n"/>
+      <c r="E67" s="10" t="n"/>
+    </row>
+    <row r="69" ht="45" customHeight="1">
+      <c r="A69" s="11" t="inlineStr">
         <is>
           <t>NOTA: Contagem feita a partir das fotografias, cada item contado uma só vez (as fotos são vários ângulos do mesmo material). Itens marcados '(aprox.)' estão empilhados ou parcialmente tapados — confirmar fisicamente. Todo o material está em embalagem estéril e original.</t>
         </is>
@@ -1650,9 +1711,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A67:B67"/>
+    <mergeCell ref="A69:E69"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A63:B63"/>
-    <mergeCell ref="A65:E65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>